<commit_message>
fix: harden weekly production manifest and completeness
</commit_message>
<xml_diff>
--- a/data/processed/production/weekly_report_2026-06-w4.xlsx
+++ b/data/processed/production/weekly_report_2026-06-w4.xlsx
@@ -5540,7 +5540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5582,12 +5582,24 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>manifest_hash</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>7895152a4306f9fa25ee42953236540cd6af1365c3e16fd2e8a06c97203cc539</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>business_fingerprint</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ab68f05858dcc312e2b76834f7c3f05d801ddeecbb7e9163b132da772e914dbe</t>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>7f57bb892f17faeb4295ddba7c5c84a619a21f9492cb3938306eb2ca04e99909</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ralph(v3): weekly-report-production-pipeline round 3
Ralph-Run-ID: weekly-report-production-20260917-r5
Ralph-Round: 3
Ralph-Task-ID: weekly-report-production-pipeline
</commit_message>
<xml_diff>
--- a/data/processed/production/weekly_report_2026-06-w4.xlsx
+++ b/data/processed/production/weekly_report_2026-06-w4.xlsx
@@ -5587,7 +5587,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7895152a4306f9fa25ee42953236540cd6af1365c3e16fd2e8a06c97203cc539</t>
+          <t>7a6d0637e5b6ead248912d9f00472bba8b1edaf1f377d9c69be7d1ce8b88d5d3</t>
         </is>
       </c>
     </row>
@@ -5599,7 +5599,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7f57bb892f17faeb4295ddba7c5c84a619a21f9492cb3938306eb2ca04e99909</t>
+          <t>f7895ecc16a7298fbb9da7e58fa6a641106157f6077d637b52fa24e3cadd60a2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ralph(v3): weekly-report-production-pipeline round 5
Ralph-Run-ID: weekly-report-production-20260917-r5
Ralph-Round: 5
Ralph-Task-ID: weekly-report-production-pipeline
</commit_message>
<xml_diff>
--- a/data/processed/production/weekly_report_2026-06-w4.xlsx
+++ b/data/processed/production/weekly_report_2026-06-w4.xlsx
@@ -909,7 +909,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>f7895ecc16a7298fbb9da7e58fa6a641106157f6077d637b52fa24e3cadd60a2</t>
+          <t>3904d6560dd3061cf69dc6281c57fbe65bbe7a858e2a2115008251d761c6f52a</t>
         </is>
       </c>
     </row>
@@ -1280,48 +1280,6 @@
           <t>月  总</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>263</v>
-      </c>
-      <c r="C9" t="n">
-        <v>57</v>
-      </c>
-      <c r="D9" t="n">
-        <v>37</v>
-      </c>
-      <c r="E9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" t="n">
-        <v>13</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" t="n">
-        <v>130</v>
-      </c>
-      <c r="K9" t="n">
-        <v>39</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>17</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>39</v>
-      </c>
     </row>
     <row r="10"/>
     <row r="11">
@@ -1330,20 +1288,8 @@
           <t>当周</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>263</v>
-      </c>
-      <c r="C11" t="n">
-        <v>57</v>
-      </c>
-      <c r="D11" t="n">
-        <v>37</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2</v>
-      </c>
       <c r="F11" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -1351,26 +1297,14 @@
       <c r="H11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="n">
-        <v>130</v>
-      </c>
-      <c r="K11" t="n">
-        <v>39</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
       <c r="M11" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>1</v>
       </c>
       <c r="O11" t="n">
         <v>4</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1708,7 +1642,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
         <v>6</v>
@@ -1717,7 +1651,7 @@
         <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -1754,7 +1688,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
         <v>9</v>
@@ -1763,7 +1697,7 @@
         <v>2.25</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G5" t="n">
         <v>3</v>
@@ -1809,7 +1743,7 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
@@ -1846,7 +1780,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>9</v>
@@ -1855,7 +1789,7 @@
         <v>2.25</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
@@ -1892,7 +1826,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
         <v>12</v>
@@ -1938,7 +1872,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D9" t="n">
         <v>12</v>
@@ -1947,7 +1881,7 @@
         <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
@@ -1984,7 +1918,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
         <v>12</v>
@@ -2030,7 +1964,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D11" t="n">
         <v>12</v>
@@ -2039,7 +1973,7 @@
         <v>1.5</v>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -2260,7 +2194,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
         <v>9</v>
@@ -2269,7 +2203,7 @@
         <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G16" t="n">
         <v>5</v>
@@ -2306,7 +2240,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
         <v>12</v>
@@ -2315,7 +2249,7 @@
         <v>2.4</v>
       </c>
       <c r="F17" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G17" t="n">
         <v>4</v>
@@ -2398,7 +2332,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
         <v>6</v>
@@ -2407,7 +2341,7 @@
         <v>1.5</v>
       </c>
       <c r="F19" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G19" t="n">
         <v>6</v>
@@ -2444,7 +2378,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" t="n">
         <v>12</v>
@@ -2490,7 +2424,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
         <v>9</v>
@@ -2693,23 +2627,17 @@
       <c r="C7" t="n">
         <v>356</v>
       </c>
-      <c r="D7" t="n">
-        <v>2180.5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>356</v>
-      </c>
       <c r="H7" t="n">
-        <v>219</v>
+        <v>94</v>
       </c>
       <c r="I7" t="n">
         <v>219</v>
       </c>
       <c r="L7" t="n">
-        <v>411</v>
+        <v>169</v>
       </c>
       <c r="M7" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="N7" t="n">
         <v>411</v>
@@ -2723,59 +2651,23 @@
       <c r="B9" t="n">
         <v>2180.5</v>
       </c>
-      <c r="C9" t="n">
-        <v>356</v>
-      </c>
-      <c r="D9" t="n">
-        <v>2180.5</v>
-      </c>
-      <c r="E9" t="n">
-        <v>356</v>
-      </c>
-      <c r="H9" t="n">
-        <v>219</v>
-      </c>
-      <c r="I9" t="n">
-        <v>219</v>
-      </c>
-      <c r="L9" t="n">
-        <v>411</v>
-      </c>
-      <c r="M9" t="n">
-        <v>18</v>
-      </c>
-      <c r="N9" t="n">
-        <v>411</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="10"/>
     <row r="11">
-      <c r="B11" t="n">
-        <v>2180.5</v>
-      </c>
       <c r="C11" t="n">
         <v>356</v>
       </c>
-      <c r="D11" t="n">
-        <v>2180.5</v>
-      </c>
-      <c r="E11" t="n">
-        <v>356</v>
-      </c>
       <c r="H11" t="n">
-        <v>219</v>
+        <v>94</v>
       </c>
       <c r="I11" t="n">
         <v>219</v>
       </c>
       <c r="L11" t="n">
-        <v>411</v>
+        <v>169</v>
       </c>
       <c r="M11" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="N11" t="n">
         <v>411</v>

</xml_diff>